<commit_message>
Add new PDF files for eflviewer with updated content and metadata
- Created 'eflviewer (5).pdf' with new images and form data.
- Created 'eflviewer.pdf' with updated images and form action.
- Both files include necessary metadata and structure for proper rendering.
</commit_message>
<xml_diff>
--- a/verify_results_fixed/Plan_Comparison_Summary.xlsx
+++ b/verify_results_fixed/Plan_Comparison_Summary.xlsx
@@ -15,7 +15,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+  <si>
+    <t>Price Rank</t>
+  </si>
   <si>
     <t>Company Name</t>
   </si>
@@ -23,6 +26,9 @@
     <t>Plan Name</t>
   </si>
   <si>
+    <t>Total Simulated Bill ($)</t>
+  </si>
+  <si>
     <t>Product Type</t>
   </si>
   <si>
@@ -44,9 +50,6 @@
     <t>Termination Fee ($)</t>
   </si>
   <si>
-    <t>Renewable %</t>
-  </si>
-  <si>
     <t>Time-of-Use</t>
   </si>
   <si>
@@ -56,58 +59,58 @@
     <t>CleanSky Energy</t>
   </si>
   <si>
+    <t>Free Weekends 12 - Time Of Use</t>
+  </si>
+  <si>
+    <t>Time Of Use</t>
+  </si>
+  <si>
+    <t>2 rates</t>
+  </si>
+  <si>
+    <t>Autopay required or recommended; Pricing assumes 35% of consumption during Designated Free Period</t>
+  </si>
+  <si>
+    <t>Affordable Wind 12 - Fixed</t>
+  </si>
+  <si>
+    <t>Fixed</t>
+  </si>
+  <si>
+    <t>0 rates</t>
+  </si>
+  <si>
+    <t>Autopay required or recommended; Some locations may be subject to Underground Facilities and Cost Recovery Charge</t>
+  </si>
+  <si>
+    <t>Embrace Green 24 - Fixed</t>
+  </si>
+  <si>
+    <t>Ultra Clean Solar 24 - Fixed</t>
+  </si>
+  <si>
+    <t>Embrace Green 36 - Fixed</t>
+  </si>
+  <si>
     <t>Free Month 12 - Fixed</t>
   </si>
   <si>
-    <t>Fixed</t>
-  </si>
-  <si>
-    <t>0 rates</t>
-  </si>
-  <si>
-    <t>Autopay required or recommended; Some locations may be subject to Underground Facilities and Cost Recovery Charge; 100% renewable energy content</t>
-  </si>
-  <si>
-    <t>Free Weekends 12 - Time Of Use</t>
-  </si>
-  <si>
-    <t>Time Of Use</t>
-  </si>
-  <si>
-    <t>2 rates</t>
-  </si>
-  <si>
-    <t>Autopay required or recommended; Pricing assumes 35% of consumption during Designated Free Period; 100% renewable energy content</t>
+    <t>Embrace Green 12 - Fixed</t>
+  </si>
+  <si>
+    <t>Embrace Green 6 - Fixed</t>
   </si>
   <si>
     <t>Happy Hour Power 12 - Time Of Use</t>
   </si>
   <si>
+    <t>Eco Rewards 36 - Fixed</t>
+  </si>
+  <si>
     <t>Free Nights 12 - Time Of Use</t>
   </si>
   <si>
-    <t>Autopay required or recommended; 100% renewable energy content</t>
-  </si>
-  <si>
-    <t>Eco Rewards 36 - Fixed</t>
-  </si>
-  <si>
-    <t>Ultra Clean Solar 24 - Fixed</t>
-  </si>
-  <si>
-    <t>Affordable Wind 12 - Fixed</t>
-  </si>
-  <si>
-    <t>Embrace Green 12 - Fixed</t>
-  </si>
-  <si>
-    <t>Embrace Green 6 - Fixed</t>
-  </si>
-  <si>
-    <t>Embrace Green 36 - Fixed</t>
-  </si>
-  <si>
-    <t>Embrace Green 24 - Fixed</t>
+    <t>Autopay required or recommended</t>
   </si>
   <si>
     <t>Eco Rewards 24 - Fixed</t>
@@ -525,16 +528,17 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col customWidth="true" max="1" min="1" width="15"/>
-    <col customWidth="true" max="2" min="2" width="25"/>
-    <col customWidth="true" max="4" min="3" width="15"/>
-    <col customWidth="true" max="5" min="5" width="18"/>
-    <col customWidth="true" max="6" min="6" width="15"/>
-    <col customWidth="true" max="8" min="7" width="18"/>
-    <col customWidth="true" max="9" min="9" width="15"/>
-    <col customWidth="true" max="10" min="10" width="12"/>
-    <col customWidth="true" max="11" min="11" width="20"/>
-    <col customWidth="true" max="12" min="12" width="40"/>
+    <col customWidth="true" max="1" min="1" width="10"/>
+    <col customWidth="true" max="2" min="2" width="15"/>
+    <col customWidth="true" max="3" min="3" width="28"/>
+    <col customWidth="true" max="4" min="4" width="22"/>
+    <col customWidth="true" max="6" min="5" width="15"/>
+    <col customWidth="true" max="7" min="7" width="18"/>
+    <col customWidth="true" max="8" min="8" width="15"/>
+    <col customWidth="true" max="10" min="9" width="18"/>
+    <col customWidth="true" max="11" min="11" width="15"/>
+    <col customWidth="true" max="12" min="12" width="20"/>
+    <col customWidth="true" max="13" min="13" width="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -574,10 +578,13 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
-        <v>12</v>
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
@@ -586,487 +593,526 @@
         <v>14</v>
       </c>
       <c r="D2">
+        <v>894.98</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2">
         <v>12</v>
       </c>
-      <c r="E2">
-        <v>7.9</v>
-      </c>
-      <c r="F2">
+      <c r="G2">
+        <v>16.9</v>
+      </c>
+      <c r="H2">
         <v>0</v>
       </c>
-      <c r="G2">
+      <c r="I2">
         <v>4.06</v>
       </c>
-      <c r="H2">
+      <c r="J2">
         <v>6.1196</v>
       </c>
-      <c r="I2">
+      <c r="K2">
         <v>150</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2" t="s">
-        <v>15</v>
       </c>
       <c r="L2" t="s">
         <v>16</v>
       </c>
+      <c r="M2" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="s">
-        <v>12</v>
+      <c r="A3">
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
         <v>18</v>
       </c>
       <c r="D3">
+        <v>965</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3">
         <v>12</v>
       </c>
-      <c r="E3">
-        <v>16.9</v>
-      </c>
-      <c r="F3">
+      <c r="G3">
+        <v>7.5</v>
+      </c>
+      <c r="H3">
         <v>0</v>
       </c>
-      <c r="G3">
+      <c r="I3">
         <v>4.06</v>
       </c>
-      <c r="H3">
+      <c r="J3">
         <v>6.1196</v>
       </c>
-      <c r="I3">
+      <c r="K3">
         <v>150</v>
-      </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
-      <c r="K3" t="s">
-        <v>19</v>
       </c>
       <c r="L3" t="s">
         <v>20</v>
       </c>
+      <c r="M3" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="s">
-        <v>12</v>
+      <c r="A4">
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D4">
-        <v>12</v>
-      </c>
-      <c r="E4">
-        <v>21.5</v>
+        <v>965</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
       </c>
       <c r="F4">
+        <v>24</v>
+      </c>
+      <c r="G4">
+        <v>7.5</v>
+      </c>
+      <c r="H4">
         <v>0</v>
       </c>
-      <c r="G4">
+      <c r="I4">
         <v>4.06</v>
       </c>
-      <c r="H4">
+      <c r="J4">
         <v>6.1196</v>
       </c>
-      <c r="I4">
-        <v>150</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4" t="s">
-        <v>19</v>
+      <c r="K4">
+        <v>225</v>
       </c>
       <c r="L4" t="s">
         <v>20</v>
       </c>
+      <c r="M4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="s">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5">
+        <v>971.9</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5">
+        <v>24</v>
+      </c>
+      <c r="G5">
+        <v>7.6</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>4.06</v>
+      </c>
+      <c r="J5">
+        <v>6.1196</v>
+      </c>
+      <c r="K5">
+        <v>225</v>
+      </c>
+      <c r="L5" t="s">
+        <v>20</v>
+      </c>
+      <c r="M5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6">
+        <v>985.71</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6">
+        <v>36</v>
+      </c>
+      <c r="G6">
+        <v>7.8</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>4.06</v>
+      </c>
+      <c r="J6">
+        <v>6.1196</v>
+      </c>
+      <c r="K6">
+        <v>275</v>
+      </c>
+      <c r="L6" t="s">
+        <v>20</v>
+      </c>
+      <c r="M6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7">
+        <v>992.61</v>
+      </c>
+      <c r="E7" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7">
         <v>12</v>
       </c>
-      <c r="B5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5">
+      <c r="G7">
+        <v>7.9</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <v>4.06</v>
+      </c>
+      <c r="J7">
+        <v>6.1196</v>
+      </c>
+      <c r="K7">
+        <v>150</v>
+      </c>
+      <c r="L7" t="s">
+        <v>20</v>
+      </c>
+      <c r="M7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8">
+        <v>999.51</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8">
         <v>12</v>
       </c>
-      <c r="E5">
-        <v>18.1</v>
-      </c>
-      <c r="F5">
+      <c r="G8">
+        <v>8</v>
+      </c>
+      <c r="H8">
         <v>0</v>
       </c>
-      <c r="G5">
+      <c r="I8">
         <v>4.06</v>
       </c>
-      <c r="H5">
+      <c r="J8">
         <v>6.1196</v>
       </c>
-      <c r="I5">
+      <c r="K8">
         <v>150</v>
       </c>
-      <c r="J5">
+      <c r="L8" t="s">
+        <v>20</v>
+      </c>
+      <c r="M8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9">
+        <v>999.51</v>
+      </c>
+      <c r="E9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9">
+        <v>6</v>
+      </c>
+      <c r="G9">
+        <v>8</v>
+      </c>
+      <c r="H9">
         <v>0</v>
       </c>
-      <c r="K5" t="s">
-        <v>19</v>
-      </c>
-      <c r="L5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
+      <c r="I9">
+        <v>4.06</v>
+      </c>
+      <c r="J9">
+        <v>6.1196</v>
+      </c>
+      <c r="K9">
+        <v>75</v>
+      </c>
+      <c r="L9" t="s">
+        <v>20</v>
+      </c>
+      <c r="M9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10">
+        <v>1016.85</v>
+      </c>
+      <c r="E10" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6">
-        <v>36</v>
-      </c>
-      <c r="E6">
-        <v>9.3</v>
-      </c>
-      <c r="F6">
+      <c r="G10">
+        <v>21.5</v>
+      </c>
+      <c r="H10">
         <v>0</v>
       </c>
-      <c r="G6">
+      <c r="I10">
         <v>4.06</v>
       </c>
-      <c r="H6">
+      <c r="J10">
         <v>6.1196</v>
       </c>
-      <c r="I6">
-        <v>275</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6" t="s">
-        <v>15</v>
-      </c>
-      <c r="L6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>25</v>
-      </c>
-      <c r="C7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7">
-        <v>24</v>
-      </c>
-      <c r="E7">
-        <v>7.6</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>4.06</v>
-      </c>
-      <c r="H7">
-        <v>6.1196</v>
-      </c>
-      <c r="I7">
-        <v>225</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7" t="s">
-        <v>15</v>
-      </c>
-      <c r="L7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8">
-        <v>12</v>
-      </c>
-      <c r="E8">
-        <v>7.5</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8">
-        <v>4.06</v>
-      </c>
-      <c r="H8">
-        <v>6.1196</v>
-      </c>
-      <c r="I8">
+      <c r="K10">
         <v>150</v>
-      </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8" t="s">
-        <v>15</v>
-      </c>
-      <c r="L8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9">
-        <v>12</v>
-      </c>
-      <c r="E9">
-        <v>8</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>4.06</v>
-      </c>
-      <c r="H9">
-        <v>6.1196</v>
-      </c>
-      <c r="I9">
-        <v>150</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9" t="s">
-        <v>15</v>
-      </c>
-      <c r="L9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10">
-        <v>6</v>
-      </c>
-      <c r="E10">
-        <v>8</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-      <c r="G10">
-        <v>4.06</v>
-      </c>
-      <c r="H10">
-        <v>6.1196</v>
-      </c>
-      <c r="I10">
-        <v>75</v>
-      </c>
-      <c r="J10">
-        <v>0</v>
-      </c>
-      <c r="K10" t="s">
-        <v>15</v>
       </c>
       <c r="L10" t="s">
         <v>16</v>
       </c>
+      <c r="M10" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="s">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11">
+        <v>1089.26</v>
+      </c>
+      <c r="E11" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11">
+        <v>36</v>
+      </c>
+      <c r="G11">
+        <v>9.3</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>4.06</v>
+      </c>
+      <c r="J11">
+        <v>6.1196</v>
+      </c>
+      <c r="K11">
+        <v>275</v>
+      </c>
+      <c r="L11" t="s">
+        <v>20</v>
+      </c>
+      <c r="M11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12">
+        <v>1262.25</v>
+      </c>
+      <c r="E12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12">
         <v>12</v>
       </c>
-      <c r="B11" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11">
-        <v>36</v>
-      </c>
-      <c r="E11">
-        <v>7.8</v>
-      </c>
-      <c r="F11">
+      <c r="G12">
+        <v>18.1</v>
+      </c>
+      <c r="H12">
         <v>0</v>
       </c>
-      <c r="G11">
+      <c r="I12">
         <v>4.06</v>
       </c>
-      <c r="H11">
+      <c r="J12">
         <v>6.1196</v>
       </c>
-      <c r="I11">
-        <v>275</v>
-      </c>
-      <c r="J11">
-        <v>0</v>
-      </c>
-      <c r="K11" t="s">
-        <v>15</v>
-      </c>
-      <c r="L11" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12">
-        <v>24</v>
-      </c>
-      <c r="E12">
-        <v>7.5</v>
-      </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
-      <c r="G12">
-        <v>4.06</v>
-      </c>
-      <c r="H12">
-        <v>6.1196</v>
-      </c>
-      <c r="I12">
-        <v>225</v>
-      </c>
-      <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12" t="s">
-        <v>15</v>
+      <c r="K12">
+        <v>150</v>
       </c>
       <c r="L12" t="s">
         <v>16</v>
       </c>
+      <c r="M12" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="s">
+      <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="D13">
+        <v>1351.59</v>
+      </c>
+      <c r="E13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13">
         <v>24</v>
       </c>
-      <c r="E13">
+      <c r="G13">
         <v>13.1</v>
       </c>
-      <c r="F13">
+      <c r="H13">
         <v>0</v>
       </c>
-      <c r="G13">
+      <c r="I13">
         <v>4.06</v>
       </c>
-      <c r="H13">
+      <c r="J13">
         <v>6.1196</v>
       </c>
-      <c r="I13">
+      <c r="K13">
         <v>225</v>
       </c>
-      <c r="J13">
+      <c r="L13" t="s">
+        <v>20</v>
+      </c>
+      <c r="M13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14">
+        <v>1351.59</v>
+      </c>
+      <c r="E14" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14">
+        <v>24</v>
+      </c>
+      <c r="G14">
+        <v>13.1</v>
+      </c>
+      <c r="H14">
         <v>0</v>
       </c>
-      <c r="K13" t="s">
-        <v>15</v>
-      </c>
-      <c r="L13" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14">
-        <v>24</v>
-      </c>
-      <c r="E14">
-        <v>13.1</v>
-      </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
-      <c r="G14">
+      <c r="I14">
         <v>4.06</v>
       </c>
-      <c r="H14">
+      <c r="J14">
         <v>6.1196</v>
       </c>
-      <c r="I14">
+      <c r="K14">
         <v>225</v>
       </c>
-      <c r="J14">
-        <v>0</v>
-      </c>
-      <c r="K14" t="s">
-        <v>15</v>
-      </c>
       <c r="L14" t="s">
-        <v>16</v>
+        <v>20</v>
+      </c>
+      <c r="M14" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1083,986 +1129,986 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11"/>
     <row r="12"/>
     <row r="13">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B18" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C20" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C21" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26"/>
     <row r="27"/>
     <row r="28">
       <c r="A28" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B29" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B30" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B31" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B32" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B33" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B35" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B36" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C36" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="41"/>
     <row r="42"/>
     <row r="43">
       <c r="A43" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B43" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B44" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B45" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B46" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B47" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B48" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B50" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C50" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B51" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C51" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="55"/>
     <row r="56"/>
     <row r="57">
       <c r="A57" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B57" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B58" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B59" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B60" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B61" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B62" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="67"/>
     <row r="68"/>
     <row r="69">
       <c r="A69" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B69" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B70" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B71" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B72" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B73" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B74" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="79"/>
     <row r="80"/>
     <row r="81">
       <c r="A81" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B81" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B82" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B83" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B84" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B85" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B86" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="91"/>
     <row r="92"/>
     <row r="93">
       <c r="A93" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B93" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B94" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B95" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B96" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B97" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B98" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="103"/>
     <row r="104"/>
     <row r="105">
       <c r="A105" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B105" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B106" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B107" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B108" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B109" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B110" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="115"/>
     <row r="116"/>
     <row r="117">
       <c r="A117" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B117" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B118" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B119" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B120" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B121" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B122" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="127"/>
     <row r="128"/>
     <row r="129">
       <c r="A129" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B129" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B130" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B131" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B132" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B133" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B134" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="139"/>
     <row r="140"/>
     <row r="141">
       <c r="A141" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B141" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B142" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B143" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B144" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B145" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B146" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="151"/>
     <row r="152"/>
     <row r="153">
       <c r="A153" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B153" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B154" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B155" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B156" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B157" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B158" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>